<commit_message>
Versjon 2.3.3 · kostnadsstrukturen hos Nordlys
Underentreprenører 3 660 000 er blitt innleide montører 400 000, lønnskostnaden 10 660 000 og bruttofortjenesten 62,5 % i hele appen: kapittel 2, 3, 4, 5, 6 og 9, markedsføring 5 og organisasjon 18, med nytt budsjett og likviditetsbudsjett for 2027. Pensumfiler (PDF og regneark) speilet fra LOM_Pensum_2026_v3.
</commit_message>
<xml_diff>
--- a/pensum/ma03/LOM_Ovingsark_Markedsforing_kap03_Markedsbudsjett_NY.xlsx
+++ b/pensum/ma03/LOM_Ovingsark_Markedsforing_kap03_Markedsbudsjett_NY.xlsx
@@ -2249,7 +2249,7 @@
     </row>
     <row r="29">
       <c r="A29" s="20" t="n">
-        <v>0.48</v>
+        <v>0.625</v>
       </c>
       <c r="B29" s="16">
         <f>Budsjett!$D$31/A29</f>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Omsetning minus materiell, underentreprenører og de timene som går med.</t>
+          <t>Omsetning minus materiell, innleide montører og de timene som går med.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Versjon 2.5.1 · kildeavvik og boknavn rettet
</commit_message>
<xml_diff>
--- a/pensum/ma03/LOM_Ovingsark_Markedsforing_kap03_Markedsbudsjett_NY.xlsx
+++ b/pensum/ma03/LOM_Ovingsark_Markedsforing_kap03_Markedsbudsjett_NY.xlsx
@@ -300,7 +300,7 @@
     <t xml:space="preserve">Kilder</t>
   </si>
   <si>
-    <t xml:space="preserve">Hjertnes, F.: Markedsføring, organisasjon og ledelse for LØM-emnet, 4. utg., kap. 3.3 til 3.6. Nullpunktstankegangen er den samme som i Bok 1 Økonomistyring kap. 8.</t>
+    <t xml:space="preserve">Hjertnes, F.: Markedsføring, organisasjon og ledelse for LØM-emnet, 4. utg., kap. 3.3 til 3.6. Nullpunktstankegangen er den samme som i Økonomistyring for LØM-emnet, kap. 8.</t>
   </si>
   <si>
     <t xml:space="preserve">Markedstall: NVE, «Solkraft», nve.no/energi/energisystem/solkraft (tall per 31.12.2024, hentet 09.09.2026) og SSB, statistikken «Bilparken», publisert 06.03.2026 (tall per 31.12.2025, hentet 09.09.2026).</t>
@@ -585,7 +585,7 @@
     <t xml:space="preserve">Prøv dette: sett dekningsgraden opp ved å heve dekningsbidraget per ladepunkt i Budsjett!B13, og se hvor mye mindre omsetning som må til.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kilde: nullpunktstankegangen er den samme som i Bok 1 Økonomistyring kap. 8. Markedsbudsjettet hører til markedsplanens siste ledd, Hjertnes kap. 3.5.</t>
+    <t xml:space="preserve">Kilde: nullpunktstankegangen er den samme som i Økonomistyring for LØM-emnet, kap. 8. Markedsbudsjettet hører til markedsplanens siste ledd, Hjertnes kap. 3.5.</t>
   </si>
   <si>
     <t xml:space="preserve">Tre scenarioer</t>
@@ -735,7 +735,7 @@
     <t xml:space="preserve">Er det margin igjen?</t>
   </si>
   <si>
-    <t xml:space="preserve">Kilde: Hjertnes kap. 3.4 og 3.5. Nullpunktstankegangen er den samme som i Bok 1 Økonomistyring kap. 8. Tallene er Nordlys Elektro AS sine egne.</t>
+    <t xml:space="preserve">Kilde: Hjertnes kap. 3.4 og 3.5. Nullpunktstankegangen er den samme som i Økonomistyring for LØM-emnet, kap. 8. Tallene er Nordlys Elektro AS sine egne.</t>
   </si>
   <si>
     <t xml:space="preserve">Din egen bedrift</t>

</xml_diff>